<commit_message>
verification(SEEPW-T07): the sample's van Genuchten pair is fit to the vendor conductivity table
The multistep-outflow example ships an 80-point retention spline and an 80-point
conductivity spline for the sample, PEST-calibrated together, and xslope carries
one (alpha, n) per material. The pair now follows the standing rule: least
squares in log10 kr against the CONDUCTIVITY table over the suction range the
run reaches. The column is hydrostatic above a base held at the stage suction,
so it reaches 0.298 m, and the live part of the vendor's curve -- its 54 points
above kr = 1e-4 -- lies entirely inside that. alpha = 8.8157 /m, n = 9.7144;
0.0033 decades rms against the table where the retention pair reads 0.055.

The docstring also records what the 1e-4 conductivity floor costs this row,
measured by re-solving with the floor lowered. No default is changed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/geostudio/gs2_mso.xlsx
+++ b/docs/verification/files/geostudio/gs2_mso.xlsx
@@ -6882,10 +6882,10 @@
         <v>-0.4</v>
       </c>
       <c r="AM11" s="3">
-        <v>8.9125</v>
+        <v>8.8157</v>
       </c>
       <c r="AN11" s="3">
-        <v>10.1875</v>
+        <v>9.7144</v>
       </c>
       <c r="AO11" s="3">
         <v>1e-05</v>
@@ -8412,9 +8412,7 @@
       <c r="A2" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="3">
-        <v>0</v>
-      </c>
+      <c r="B2" s="3"/>
       <c r="D2" s="24" t="s">
         <v>147</v>
       </c>

</xml_diff>

<commit_message>
verification(geostudio): T07 carries SEEP/W's own van Genuchten and Mualem parameters
Both of the vendor's 80-point splines for the sample are closed forms
tabulated at 80 points, not measurements, so the builder reads the parameters
back out of them instead of fitting the law to one table at the other's
expense: van Genuchten (alpha, n) against all 80 retention points closes to
2.3e-10 rms in water content, and the Mualem exponent l against the 56
conductivity points above kr = 1e-6 to 1.9e-7 rms in decades. alpha = 8.893966
/m, n = 10.190410, l = 0.295141, with theta_r = 0.0290384 the table's own dry
plateau. Fitting all three to the conductivity table together returns the same
numbers.

Under Mualem's l = 0.5 no single pair reproduces both curves, which is what
the shipped fit-to-conductivity pair was paying for.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/geostudio/gs2_mso.xlsx
+++ b/docs/verification/files/geostudio/gs2_mso.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523500CF-89B8-4644-B955-31C74218CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12967D2-A998-D342-B5ED-43CABE326A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15680" yWindow="4780" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="319">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t>vg</t>
-  </si>
-  <si>
-    <t>van Genuchten model (a, n)</t>
   </si>
   <si>
     <t>pow</t>
@@ -1134,6 +1131,12 @@
   </si>
   <si>
     <t>Unrotated</t>
+  </si>
+  <si>
+    <t>van Genuchten model (a, n, l)</t>
+  </si>
+  <si>
+    <t>l</t>
   </si>
 </sst>
 </file>
@@ -2881,7 +2884,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3061,7 +3064,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>46</v>
@@ -3156,7 +3159,7 @@
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D58" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
@@ -3298,73 +3301,73 @@
   <sheetData>
     <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>246</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="H2" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="I2" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="J2" s="27" t="s">
         <v>249</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="L2" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="M2" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="O2" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="M2" s="27" t="s">
-        <v>311</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>312</v>
-      </c>
-      <c r="O2" s="27" t="s">
+      <c r="P2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="P2" s="27" t="s">
+      <c r="Q2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="Q2" s="27" t="s">
+      <c r="R2" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="S2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="T2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="S2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="T2" s="28" t="s">
+      <c r="AB2" t="s">
         <v>257</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>258</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>259</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.2">
@@ -3397,13 +3400,13 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="AB3" t="s">
+        <v>260</v>
+      </c>
+      <c r="AC3" t="s">
         <v>261</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>262</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.2">
@@ -3436,7 +3439,7 @@
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="AB4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
@@ -3469,7 +3472,7 @@
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="AB5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.2">
@@ -3562,13 +3565,13 @@
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
       <c r="AB8" t="s">
+        <v>257</v>
+      </c>
+      <c r="AC8" t="s">
         <v>258</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AD8" t="s">
         <v>259</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.2">
@@ -3601,13 +3604,13 @@
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="AB9" t="s">
+        <v>260</v>
+      </c>
+      <c r="AC9" t="s">
         <v>261</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AD9" t="s">
         <v>262</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.2">
@@ -3640,13 +3643,13 @@
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="AB10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AC10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AD10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.2">
@@ -3679,13 +3682,13 @@
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="AB11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AC11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AD11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.2">
@@ -4029,7 +4032,7 @@
       <c r="L24" s="9"/>
       <c r="V24" s="26"/>
       <c r="W24" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
@@ -4037,7 +4040,7 @@
       <c r="L25" s="9"/>
       <c r="V25" s="29"/>
       <c r="W25" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4072,61 +4075,61 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>246</v>
-      </c>
       <c r="G2" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="I2" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="H2" s="40" t="s">
-        <v>249</v>
-      </c>
-      <c r="I2" s="27" t="s">
+      <c r="J2" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="41" t="s">
         <v>268</v>
       </c>
-      <c r="K2" s="41" t="s">
+      <c r="L2" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="M2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="N2" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="M2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="N2" s="28" t="s">
-        <v>271</v>
-      </c>
       <c r="O2" s="28" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="P2" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q2" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="Q2" s="28" t="s">
-        <v>315</v>
-      </c>
       <c r="Z2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AA2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -4150,10 +4153,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AA3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -4177,7 +4180,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="Z4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
@@ -4201,7 +4204,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="Z5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
@@ -4364,13 +4367,13 @@
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="S16" s="26"/>
       <c r="T16" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="19:20" x14ac:dyDescent="0.2">
       <c r="S17" s="29"/>
       <c r="T17" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4399,22 +4402,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>167</v>
-      </c>
       <c r="E2" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>272</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4637,27 +4640,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4675,67 +4678,67 @@
         </is>
       </c>
       <c r="H3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4756,10 +4759,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4780,7 +4783,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -5069,27 +5072,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -5097,71 +5100,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -5178,10 +5181,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5490,16 +5493,16 @@
         </is>
       </c>
       <c r="D2" s="50" t="s">
+        <v>293</v>
+      </c>
+      <c r="E2" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>296</v>
-      </c>
-      <c r="G2" s="50" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -5514,7 +5517,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J3" s="3">
         <v>219621.96</v>
@@ -5546,7 +5549,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -5576,7 +5579,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -5592,7 +5595,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -5608,7 +5611,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -6463,16 +6466,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:AP52"/>
+  <dimension ref="A2:AQ52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="41" width="8.5" customWidth="1"/>
+    <col min="11" max="42" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>79</v>
       </c>
@@ -6487,7 +6490,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>83</v>
       </c>
@@ -6508,7 +6511,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>89</v>
       </c>
@@ -6530,67 +6533,67 @@
         <v>93</v>
       </c>
       <c r="AK4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C5" s="1" t="s">
+      <c r="D5" t="s">
         <v>95</v>
-      </c>
-      <c r="D5" t="s">
-        <v>96</v>
       </c>
       <c r="L5" s="26"/>
       <c r="M5" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="O5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="P5" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="AD5" s="14"/>
       <c r="AJ5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AK5" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="AK5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="L6" s="29"/>
       <c r="M6" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="O6" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="P6" t="s">
         <v>105</v>
-      </c>
-      <c r="P6" t="s">
-        <v>106</v>
       </c>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C9" s="53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="52"/>
@@ -6616,7 +6619,7 @@
       <c r="Y9" s="54"/>
       <c r="Z9" s="54"/>
       <c r="AA9" s="53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -6624,7 +6627,7 @@
       <c r="AE9" s="54"/>
       <c r="AF9" s="54"/>
       <c r="AG9" s="53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH9" s="54"/>
       <c r="AI9" s="54"/>
@@ -6635,136 +6638,140 @@
       <c r="AN9" s="54"/>
       <c r="AO9" s="54"/>
       <c r="AP9" s="54"/>
-    </row>
-    <row r="10" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AQ9" s="54"/>
+    </row>
+    <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="45" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="D10" s="48" t="s">
+        <v>308</v>
+      </c>
+      <c r="E10" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="E10" s="44" t="s">
+      <c r="F10" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="G10" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="45" t="s">
+      <c r="H10" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="I10" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="I10" s="44" t="s">
+      <c r="J10" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="J10" s="49" t="s">
+      <c r="K10" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="K10" s="49" t="s">
+      <c r="L10" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="M10" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="N10" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="O10" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="O10" s="44" t="s">
+      <c r="P10" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="P10" s="44" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q10" s="44" t="s">
+      <c r="R10" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="R10" s="44" t="s">
+      <c r="S10" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="S10" s="44" t="s">
+      <c r="T10" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="T10" s="44" t="s">
+      <c r="U10" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="U10" s="44" t="s">
+      <c r="V10" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="V10" s="44" t="s">
+      <c r="W10" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="W10" s="44" t="s">
+      <c r="X10" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="X10" s="44" t="s">
+      <c r="Y10" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="Y10" s="44" t="s">
+      <c r="Z10" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="Z10" s="44" t="s">
+      <c r="AA10" s="46" t="s">
+        <v>304</v>
+      </c>
+      <c r="AB10" s="46" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC10" s="47" t="s">
         <v>134</v>
       </c>
-      <c r="AA10" s="46" t="s">
+      <c r="AD10" s="46" t="s">
         <v>305</v>
       </c>
-      <c r="AB10" s="46" t="s">
-        <v>304</v>
-      </c>
-      <c r="AC10" s="47" t="s">
+      <c r="AE10" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="AD10" s="46" t="s">
-        <v>306</v>
-      </c>
-      <c r="AE10" s="46" t="s">
-        <v>307</v>
-      </c>
-      <c r="AF10" s="47" t="s">
-        <v>308</v>
-      </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AI10" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="AM10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AN10" s="23" t="s">
+      <c r="AO10" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="AP10" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AO10" s="23" t="s">
+      <c r="AQ10" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AP10" s="23" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -6882,19 +6889,22 @@
         <v>-0.4</v>
       </c>
       <c r="AM11" s="3">
-        <v>8.8157</v>
+        <v>8.893966</v>
       </c>
       <c r="AN11" s="3">
-        <v>9.7144</v>
+        <v>10.19041</v>
       </c>
       <c r="AO11" s="3">
+        <v>0.295141</v>
+      </c>
+      <c r="AP11" s="3">
         <v>1e-05</v>
       </c>
-      <c r="AP11" s="3">
-        <v>0.319</v>
-      </c>
-    </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ11" s="3">
+        <v>0.3189616</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -7018,13 +7028,16 @@
         <v>0.0</v>
       </c>
       <c r="AO12" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="AP12" s="19">
         <v>1e-05</v>
       </c>
-      <c r="AP12" s="19">
+      <c r="AQ12" s="19">
         <v>0.01</v>
       </c>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -7069,8 +7082,9 @@
       <c r="AN13" s="19"/>
       <c r="AO13" s="19"/>
       <c r="AP13" s="19"/>
-    </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ13" s="19"/>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -7115,8 +7129,9 @@
       <c r="AN14" s="3"/>
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
-    </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ14" s="3"/>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -7161,8 +7176,9 @@
       <c r="AN15" s="3"/>
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
-    </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ15" s="3"/>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -7207,8 +7223,9 @@
       <c r="AN16" s="3"/>
       <c r="AO16" s="3"/>
       <c r="AP16" s="3"/>
-    </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ16" s="3"/>
+    </row>
+    <row r="17" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -7253,8 +7270,9 @@
       <c r="AN17" s="3"/>
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
-    </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ17" s="3"/>
+    </row>
+    <row r="18" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -7299,8 +7317,9 @@
       <c r="AN18" s="3"/>
       <c r="AO18" s="3"/>
       <c r="AP18" s="3"/>
-    </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ18" s="3"/>
+    </row>
+    <row r="19" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -7345,8 +7364,9 @@
       <c r="AN19" s="3"/>
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
-    </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ19" s="3"/>
+    </row>
+    <row r="20" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -7391,8 +7411,9 @@
       <c r="AN20" s="3"/>
       <c r="AO20" s="3"/>
       <c r="AP20" s="3"/>
-    </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ20" s="3"/>
+    </row>
+    <row r="21" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -7437,8 +7458,9 @@
       <c r="AN21" s="3"/>
       <c r="AO21" s="3"/>
       <c r="AP21" s="3"/>
-    </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ21" s="3"/>
+    </row>
+    <row r="22" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -7483,8 +7505,9 @@
       <c r="AN22" s="3"/>
       <c r="AO22" s="3"/>
       <c r="AP22" s="3"/>
-    </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ22" s="3"/>
+    </row>
+    <row r="23" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -7529,8 +7552,9 @@
       <c r="AN23" s="3"/>
       <c r="AO23" s="3"/>
       <c r="AP23" s="3"/>
-    </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ23" s="3"/>
+    </row>
+    <row r="24" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -7575,8 +7599,9 @@
       <c r="AN24" s="3"/>
       <c r="AO24" s="3"/>
       <c r="AP24" s="3"/>
-    </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ24" s="3"/>
+    </row>
+    <row r="25" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -7621,8 +7646,9 @@
       <c r="AN25" s="3"/>
       <c r="AO25" s="3"/>
       <c r="AP25" s="3"/>
-    </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ25" s="3"/>
+    </row>
+    <row r="26" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -7655,8 +7681,9 @@
       <c r="AN26" s="1"/>
       <c r="AO26" s="1"/>
       <c r="AP26" s="1"/>
-    </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ26" s="1"/>
+    </row>
+    <row r="27" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -7680,7 +7707,7 @@
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -7704,7 +7731,7 @@
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -7728,7 +7755,7 @@
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -7752,7 +7779,7 @@
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -7776,7 +7803,7 @@
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -8282,7 +8309,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="AG9:AP9"/>
+    <mergeCell ref="AG9:AQ9"/>
     <mergeCell ref="AA9:AF9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
@@ -8362,7 +8389,7 @@
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
+  <conditionalFormatting sqref="AM11:AO52">
     <cfRule type="expression" dxfId="18" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
@@ -8410,181 +8437,181 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B2" s="3"/>
       <c r="D2" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="N2" s="24" t="s">
         <v>147</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -8677,172 +8704,172 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B7" s="37"/>
       <c r="D7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E7" s="37"/>
       <c r="G7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H7" s="37"/>
       <c r="J7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K7" s="37"/>
       <c r="M7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N7" s="37"/>
       <c r="P7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q7" s="37"/>
       <c r="R7" s="1"/>
       <c r="S7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="1"/>
       <c r="V7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W7" s="37"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z7" s="37"/>
       <c r="AA7" s="1"/>
       <c r="AB7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC7" s="37"/>
       <c r="AE7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF7" s="37"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI7" s="37"/>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL7" s="37"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO7" s="37"/>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR7" s="37"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM8" s="1"/>
       <c r="AN8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR8" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
@@ -9647,6 +9674,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9663,20 +9704,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9710,10 +9737,10 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>168</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
@@ -9730,69 +9757,69 @@
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
@@ -9800,7 +9827,7 @@
         </is>
       </c>
       <c r="D5" s="38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E5" s="39" t="inlineStr">
         <is>
@@ -9808,187 +9835,187 @@
         </is>
       </c>
       <c r="G5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="H5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="H5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="J5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="K5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="K5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="M5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="N5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="N5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="P5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Q5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="T5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="T5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="W5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="W5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Z5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="AC5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="AE5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AF5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AI5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AI5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AL5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AL5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AO5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AO5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AR5" s="39" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B6" s="39">
         <v>1</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E6" s="39">
         <v>2</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H6" s="39">
         <v>3</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K6" s="39">
         <v>4</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N6" s="39">
         <v>5</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q6" s="39">
         <v>6</v>
       </c>
       <c r="R6" s="1"/>
       <c r="S6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T6" s="39">
         <v>7</v>
       </c>
       <c r="U6" s="1"/>
       <c r="V6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W6" s="39">
         <v>8</v>
       </c>
       <c r="X6" s="1"/>
       <c r="Y6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z6" s="39">
         <v>9</v>
       </c>
       <c r="AA6" s="1"/>
       <c r="AB6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC6" s="39">
         <v>10</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF6" s="39">
         <v>11</v>
       </c>
       <c r="AG6" s="1"/>
       <c r="AH6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI6" s="39">
         <v>12</v>
       </c>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL6" s="39">
         <v>13</v>
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO6" s="39">
         <v>14</v>
       </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR6" s="39">
         <v>15</v>
@@ -10081,172 +10108,172 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B8" s="39"/>
       <c r="D8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E8" s="39"/>
       <c r="G8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H8" s="39"/>
       <c r="J8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K8" s="39"/>
       <c r="M8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N8" s="39"/>
       <c r="P8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="1"/>
       <c r="S8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T8" s="39"/>
       <c r="U8" s="1"/>
       <c r="V8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W8" s="39"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="39"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC8" s="39"/>
       <c r="AE8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF8" s="39"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI8" s="39"/>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL8" s="39"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO8" s="39"/>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR8" s="39"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM9" s="1"/>
       <c r="AN9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR9" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
@@ -11083,6 +11110,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -11099,20 +11140,6 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -11209,20 +11236,20 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B3" s="33" t="inlineStr">
         <is>
@@ -11230,7 +11257,7 @@
         </is>
       </c>
       <c r="D3" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E3" s="35" t="inlineStr">
         <is>
@@ -11241,19 +11268,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -11266,7 +11293,7 @@
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -11275,10 +11302,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H6" t="s">
         <v>192</v>
-      </c>
-      <c r="H6" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -11415,31 +11442,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>5</v>
@@ -11467,10 +11494,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -11485,10 +11512,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -11503,10 +11530,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K5" t="s">
         <v>206</v>
-      </c>
-      <c r="K5" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -11533,7 +11560,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -11548,7 +11575,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K8"/>
     </row>
@@ -11564,7 +11591,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K9"/>
     </row>
@@ -11580,7 +11607,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K10"/>
     </row>
@@ -11596,7 +11623,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K11"/>
     </row>
@@ -11612,31 +11639,31 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K12"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K13"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K14"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K15"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -11645,7 +11672,7 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K17"/>
     </row>
@@ -11686,16 +11713,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>221</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>5</v>
@@ -11706,10 +11733,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" t="s">
         <v>222</v>
-      </c>
-      <c r="F3" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -11717,10 +11744,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F4" t="s">
         <v>224</v>
-      </c>
-      <c r="F4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -11728,10 +11755,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" t="s">
         <v>226</v>
-      </c>
-      <c r="F5" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -11861,122 +11888,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="61" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="61" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="61" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="61" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="61" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -12410,122 +12437,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="63" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="63" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="63" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="63" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="63" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">

</xml_diff>